<commit_message>
Daily slate 2026-05-26 [auto]
</commit_message>
<xml_diff>
--- a/ui_runner/templates/graded_analysis_tabs_2026-05-24.xlsx
+++ b/ui_runner/templates/graded_analysis_tabs_2026-05-24.xlsx
@@ -471,16 +471,16 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>1917</v>
+        <v>1729</v>
       </c>
       <c r="E2" t="n">
-        <v>268</v>
+        <v>231</v>
       </c>
       <c r="F2" t="n">
-        <v>1649</v>
+        <v>1498</v>
       </c>
       <c r="G2" t="n">
-        <v>14</v>
+        <v>13.4</v>
       </c>
     </row>
     <row r="3">
@@ -500,16 +500,16 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="E3" t="n">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="F3" t="n">
         <v>30</v>
       </c>
       <c r="G3" t="n">
-        <v>58.3</v>
+        <v>58.9</v>
       </c>
     </row>
     <row r="4">
@@ -529,16 +529,16 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>66</v>
+        <v>77</v>
       </c>
       <c r="E4" t="n">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="F4" t="n">
-        <v>48</v>
+        <v>53</v>
       </c>
       <c r="G4" t="n">
-        <v>27.3</v>
+        <v>31.2</v>
       </c>
     </row>
     <row r="5">
@@ -558,16 +558,16 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>42</v>
+        <v>60</v>
       </c>
       <c r="E5" t="n">
+        <v>34</v>
+      </c>
+      <c r="F5" t="n">
         <v>26</v>
       </c>
-      <c r="F5" t="n">
-        <v>16</v>
-      </c>
       <c r="G5" t="n">
-        <v>61.9</v>
+        <v>56.7</v>
       </c>
     </row>
     <row r="6">
@@ -587,16 +587,16 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="E6" t="n">
         <v>54</v>
       </c>
       <c r="F6" t="n">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="G6" t="n">
-        <v>42.9</v>
+        <v>42.5</v>
       </c>
     </row>
     <row r="7">
@@ -616,16 +616,16 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="E7" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="F7" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G7" t="n">
-        <v>64.3</v>
+        <v>64.7</v>
       </c>
     </row>
     <row r="8">
@@ -645,16 +645,16 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>451</v>
+        <v>634</v>
       </c>
       <c r="E8" t="n">
-        <v>161</v>
+        <v>193</v>
       </c>
       <c r="F8" t="n">
-        <v>290</v>
+        <v>441</v>
       </c>
       <c r="G8" t="n">
-        <v>35.7</v>
+        <v>30.4</v>
       </c>
     </row>
     <row r="9">
@@ -674,16 +674,16 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>200</v>
+        <v>189</v>
       </c>
       <c r="E9" t="n">
-        <v>118</v>
+        <v>113</v>
       </c>
       <c r="F9" t="n">
-        <v>82</v>
+        <v>76</v>
       </c>
       <c r="G9" t="n">
-        <v>59</v>
+        <v>59.8</v>
       </c>
     </row>
     <row r="10">
@@ -703,16 +703,16 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>525</v>
+        <v>588</v>
       </c>
       <c r="E10" t="n">
-        <v>327</v>
+        <v>356</v>
       </c>
       <c r="F10" t="n">
-        <v>198</v>
+        <v>232</v>
       </c>
       <c r="G10" t="n">
-        <v>62.3</v>
+        <v>60.5</v>
       </c>
     </row>
     <row r="11">
@@ -732,16 +732,16 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>306</v>
+        <v>337</v>
       </c>
       <c r="E11" t="n">
-        <v>175</v>
+        <v>192</v>
       </c>
       <c r="F11" t="n">
-        <v>131</v>
+        <v>145</v>
       </c>
       <c r="G11" t="n">
-        <v>57.2</v>
+        <v>57</v>
       </c>
     </row>
     <row r="12">
@@ -761,16 +761,16 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>156</v>
+        <v>166</v>
       </c>
       <c r="E12" t="n">
-        <v>96</v>
+        <v>103</v>
       </c>
       <c r="F12" t="n">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="G12" t="n">
-        <v>61.5</v>
+        <v>62</v>
       </c>
     </row>
     <row r="13">
@@ -790,16 +790,16 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>473</v>
+        <v>476</v>
       </c>
       <c r="E13" t="n">
         <v>167</v>
       </c>
       <c r="F13" t="n">
-        <v>306</v>
+        <v>309</v>
       </c>
       <c r="G13" t="n">
-        <v>35.3</v>
+        <v>35.1</v>
       </c>
     </row>
     <row r="14">
@@ -819,16 +819,16 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>164</v>
+        <v>186</v>
       </c>
       <c r="E14" t="n">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="F14" t="n">
-        <v>136</v>
+        <v>156</v>
       </c>
       <c r="G14" t="n">
-        <v>17.1</v>
+        <v>16.1</v>
       </c>
     </row>
     <row r="15">
@@ -848,16 +848,16 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>196</v>
+        <v>202</v>
       </c>
       <c r="E15" t="n">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="F15" t="n">
-        <v>154</v>
+        <v>158</v>
       </c>
       <c r="G15" t="n">
-        <v>21.4</v>
+        <v>21.8</v>
       </c>
     </row>
     <row r="16">
@@ -877,16 +877,16 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="E16" t="n">
         <v>16</v>
       </c>
       <c r="F16" t="n">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="G16" t="n">
-        <v>15.4</v>
+        <v>15</v>
       </c>
     </row>
     <row r="17">
@@ -906,16 +906,16 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>2865</v>
+        <v>3301</v>
       </c>
       <c r="E17" t="n">
-        <v>490</v>
+        <v>556</v>
       </c>
       <c r="F17" t="n">
-        <v>2375</v>
+        <v>2745</v>
       </c>
       <c r="G17" t="n">
-        <v>17.1</v>
+        <v>16.8</v>
       </c>
     </row>
   </sheetData>
@@ -1154,16 +1154,16 @@
         <v>77</v>
       </c>
       <c r="R2" t="n">
-        <v>13.8</v>
+        <v>12.3</v>
       </c>
       <c r="S2" t="n">
-        <v>639</v>
+        <v>555</v>
       </c>
       <c r="T2" t="n">
-        <v>14.3</v>
+        <v>27.3</v>
       </c>
       <c r="U2" t="n">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="V2" t="n">
         <v>48.7</v>
@@ -1172,10 +1172,10 @@
         <v>39</v>
       </c>
       <c r="X2" t="n">
-        <v>32.2</v>
+        <v>28.3</v>
       </c>
       <c r="Y2" t="n">
-        <v>118</v>
+        <v>198</v>
       </c>
       <c r="Z2" t="n">
         <v>50</v>
@@ -1184,10 +1184,10 @@
         <v>6</v>
       </c>
       <c r="AB2" t="n">
-        <v>100</v>
+        <v>54.5</v>
       </c>
       <c r="AC2" t="n">
-        <v>3</v>
+        <v>11</v>
       </c>
       <c r="AD2" t="n">
         <v>100</v>
@@ -1196,10 +1196,10 @@
         <v>1</v>
       </c>
       <c r="AF2" t="n">
-        <v>39.5</v>
+        <v>40</v>
       </c>
       <c r="AG2" t="n">
-        <v>43</v>
+        <v>35</v>
       </c>
     </row>
     <row r="3">
@@ -1257,16 +1257,16 @@
         <v>55</v>
       </c>
       <c r="R3" t="n">
-        <v>25.7</v>
+        <v>31.3</v>
       </c>
       <c r="S3" t="n">
-        <v>245</v>
+        <v>147</v>
       </c>
       <c r="T3" t="n">
-        <v>33.3</v>
+        <v>50</v>
       </c>
       <c r="U3" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="V3" t="n">
         <v>29.6</v>
@@ -1275,10 +1275,10 @@
         <v>27</v>
       </c>
       <c r="X3" t="n">
-        <v>39</v>
+        <v>22.2</v>
       </c>
       <c r="Y3" t="n">
-        <v>41</v>
+        <v>135</v>
       </c>
       <c r="Z3" t="n">
         <v>50</v>
@@ -1287,10 +1287,10 @@
         <v>10</v>
       </c>
       <c r="AB3" t="n">
-        <v>25</v>
+        <v>45.5</v>
       </c>
       <c r="AC3" t="n">
-        <v>4</v>
+        <v>11</v>
       </c>
       <c r="AD3" t="n">
         <v>0</v>
@@ -1299,10 +1299,10 @@
         <v>1</v>
       </c>
       <c r="AF3" t="n">
-        <v>78.8</v>
+        <v>82.2</v>
       </c>
       <c r="AG3" t="n">
-        <v>52</v>
+        <v>45</v>
       </c>
     </row>
     <row r="4">
@@ -1336,10 +1336,10 @@
         <v>0</v>
       </c>
       <c r="R4" t="n">
-        <v>5.5</v>
+        <v>5.6</v>
       </c>
       <c r="S4" t="n">
-        <v>347</v>
+        <v>341</v>
       </c>
       <c r="T4" t="n">
         <v>0</v>
@@ -1354,10 +1354,10 @@
         <v>4</v>
       </c>
       <c r="X4" t="n">
-        <v>27.1</v>
+        <v>26.1</v>
       </c>
       <c r="Y4" t="n">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="AA4" t="n">
         <v>0</v>
@@ -1579,100 +1579,100 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>62.3</v>
+        <v>60.5</v>
       </c>
       <c r="C7" t="n">
-        <v>525</v>
+        <v>588</v>
       </c>
       <c r="D7" t="n">
-        <v>57.2</v>
+        <v>57</v>
       </c>
       <c r="E7" t="n">
-        <v>306</v>
+        <v>337</v>
       </c>
       <c r="F7" t="n">
-        <v>61.5</v>
+        <v>62</v>
       </c>
       <c r="G7" t="n">
-        <v>156</v>
+        <v>166</v>
       </c>
       <c r="H7" t="n">
-        <v>35.3</v>
+        <v>35.1</v>
       </c>
       <c r="I7" t="n">
-        <v>473</v>
+        <v>476</v>
       </c>
       <c r="J7" t="n">
-        <v>17.1</v>
+        <v>16.1</v>
       </c>
       <c r="K7" t="n">
-        <v>164</v>
+        <v>186</v>
       </c>
       <c r="L7" t="n">
-        <v>21.4</v>
+        <v>21.8</v>
       </c>
       <c r="M7" t="n">
-        <v>196</v>
+        <v>202</v>
       </c>
       <c r="N7" t="n">
-        <v>15.4</v>
+        <v>15</v>
       </c>
       <c r="O7" t="n">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="P7" t="n">
-        <v>17.1</v>
+        <v>16.8</v>
       </c>
       <c r="Q7" t="n">
-        <v>2865</v>
+        <v>3301</v>
       </c>
       <c r="R7" t="n">
-        <v>14</v>
+        <v>13.4</v>
       </c>
       <c r="S7" t="n">
-        <v>1917</v>
+        <v>1729</v>
       </c>
       <c r="T7" t="n">
-        <v>27.3</v>
+        <v>31.2</v>
       </c>
       <c r="U7" t="n">
-        <v>66</v>
+        <v>77</v>
       </c>
       <c r="V7" t="n">
-        <v>42.9</v>
+        <v>42.5</v>
       </c>
       <c r="W7" t="n">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="X7" t="n">
-        <v>35.7</v>
+        <v>30.4</v>
       </c>
       <c r="Y7" t="n">
-        <v>451</v>
+        <v>634</v>
       </c>
       <c r="Z7" t="n">
-        <v>58.3</v>
+        <v>58.9</v>
       </c>
       <c r="AA7" t="n">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="AB7" t="n">
-        <v>61.9</v>
+        <v>56.7</v>
       </c>
       <c r="AC7" t="n">
-        <v>42</v>
+        <v>60</v>
       </c>
       <c r="AD7" t="n">
-        <v>64.3</v>
+        <v>64.7</v>
       </c>
       <c r="AE7" t="n">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="AF7" t="n">
-        <v>59</v>
+        <v>59.8</v>
       </c>
       <c r="AG7" t="n">
-        <v>200</v>
+        <v>189</v>
       </c>
     </row>
   </sheetData>

</xml_diff>